<commit_message>
agrego al makefile para correr el evaluation
</commit_message>
<xml_diff>
--- a/backend/evaluation/storage/metrics.xlsx
+++ b/backend/evaluation/storage/metrics.xlsx
@@ -471,8 +471,9 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The main objective of the study in Haiti was **to assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) in Haiti before and during the COVID-19 pandemic**.
-This is stated in the abstract: "Objective. To assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) in Haiti from [time period] before and during the COVID-19 pandemic." (Page 1)</t>
+          <t>The main objective of the study in Haiti was to assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) before and during the COVID-19 pandemic. 
+This is supported by the abstract which states: "Objective. To assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) in Haiti from [time period] before and during the COVID-19 pandemic." (Page 1) 
+Additionally, the study aimed to compare health indicators at the national level in two periods: pre- and peri-COVID-19 pandemic, using two-sample t-tests for proportions and variance-weighted regression. (Page 1)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -510,7 +511,10 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The data system used for the analysis was the **Haitian Unique Health Information System (SISNU)**, which collects data that are periodically uploaded to the **District Health Information Software 2 (DHIS2)**. Specifically, the analysis relied on secondary data from **SISNU-DHIS2**. (Page 2)</t>
+          <t>The data system used for the analysis was the Haitian Unique Health Information System (Système d’Information Sanitaire Unique – SISNU in French), which collects data that are periodically uploaded to the District Health Information Software 2 (DHIS2). 
+This is supported by the text which states: "A retrospective study was conducted using data from the Haitian Unique Health Information System (Système d’Infor- mation Sanitaire Unique – SISNU in French)." (Page 2) 
+Additionally, it is mentioned that "SISNU collects data on several RMNCAH indicators that can be disaggregated by age and sex. Data collected by SISNU are periodically uploaded to the District Health Information Software 2 (DHIS2)" (Page 2). 
+The analysis was also prepared based on DHIS2 data (Page 6).</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -532,7 +536,7 @@
         <v>0.8</v>
       </c>
       <c r="H3" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="4">
@@ -549,9 +553,9 @@
       <c r="C4" t="inlineStr">
         <is>
           <t>The statistical methods applied to compare pre- and peri-COVID-19 periods were:
-1. **Two-sample t-tests for proportions**: used to compare the frequency of indicators before and during the COVID-19 pandemic.
-2. **Variance-weighted regression**: used to calculate the average absolute monthly changes in health indicators.
-These methods are mentioned in the abstract (Page 1) and the methodology section (Page 2).</t>
+1. Two-sample t-tests for proportions, which were used to compare health indicators at the national level between the two periods. (Page 1 and Page 2)
+2. Variance-weighted regression, which was used to calculate the average absolute monthly changes in health indicators between the two periods. (Page 1)
+These methods were used to assess changes in reproductive, maternal, newborn, child, and adolescent health (RMNCAH) indicators in Haiti before and during the COVID-19 pandemic.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -573,7 +577,7 @@
         <v>0.8</v>
       </c>
       <c r="H4" t="n">
-        <v>0.85</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="5">
@@ -590,11 +594,11 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>The maternal health indicators that saw the most significant decline were:
-1. **Pregnant women with four antenatal care visits**
-2. **Pregnant women with five antenatal care visits or more**
-3. **Pregnant women who received a second dose of tetanus vaccine (dT2+)**
-These indicators decreased by over 4 percentage points during the pre- and peri-COVID-19 pandemic periods. (Page 4)
-Additionally, the maternal mortality ratio showed a statistically significant increase from 195 to 230 per 100,000 live births (p = 0.0082) from the pre- to the peri-COVID-19 pandemic period. (Page 4)</t>
+1. Pregnant women with four antenatal care visits
+2. Pregnant women with five antenatal care visits or more
+3. Pregnant women who received a second dose of tetanus vaccine (dT2+)
+These indicators declined by over 4 percentage points from the pre- to the peri-COVID-19 pandemic period. 
+This is supported by the text which states: "However, the most affected indicators were the proportions of pregnant women with four antenatal care visits, with five antenatal care visits or more, and those who received a second dose of tetanus vaccine, which decreased by over 4 percentage points during the two periods." (Page 1 and Page 4)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -633,13 +637,13 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>The child vaccination indicators that declined the most were:
-1. **BCG vaccine**
-2. **Diphtheria, Tetanus, and Pertussis (DTaP) vaccine**
-3. **Polio vaccine**
-4. **Pentavalent vaccine**
-5. **Rotavirus vaccine**
-These indicators all declined by over 8 percentage points during the pre- and peri-COVID-19 pandemic periods. (Page 4)
-In contrast, the **pneumococcal conjugate vaccine** increased by over 4 percentage points. (Page 4)</t>
+1. BCG vaccine
+2. DTaP (diphtheria, tetanus, and pertussis) vaccine
+3. Polio vaccine
+4. Pentavalent vaccine
+5. Rotavirus vaccine
+These indicators all declined by over 8 percentage points from the pre- to the peri-COVID-19 pandemic period.
+This is supported by the text which states: "Likewise, the proportions of children who received diphtheria, tetanus, and pertussis (DTaP), BCG, polio, pentavalent, and rotavirus vaccines also all declined by over 8 percentage points." (Page 1 and Page 4)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -661,7 +665,7 @@
         <v>0.8</v>
       </c>
       <c r="H6" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="7">
@@ -678,10 +682,11 @@
       <c r="C7" t="inlineStr">
         <is>
           <t>The pneumococcal conjugate vaccine unexpectedly increased during the pandemic. 
-According to the text: 
-- "the pneumococcal conjugate vaccine increased by over 4 percentage points" (Page 4).
-- "the number of children who received a third dose of pneumococcal conjugate vaccine increased significantly from the pre- to the peri-COVID-19 pandemic period" (Page 4).
-- This increase might be explained by the recent introduction of the vaccine into the Government's routine immunization program (Page 5).</t>
+This is supported by the text which states: 
+* "The number of women opting for the contraceptive implant and children receiving a third dose of pneumococcal conjugate vaccine increased significantly from the pre- to the peri-COVID-19 pandemic period." (Page 4)
+* "Likewise, ... pneumococcal conjugate vaccine increased by over 4 percentage points." (Page 1)
+* "The only indicator that increased by more than 4 percentage points during the period was for pneumococcal conjugate vaccine." (Page 4)
+The increase in pneumococcal conjugate vaccine uptake may be attributed to its recent introduction into the Government's routine immunization program (Page 5).</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -720,10 +725,10 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>Maternal mortality increased during the peri-COVID-19 period. 
-The maternal mortality ratio showed a statistically significant increase from 195 to 230 per 100,000 live births (p = 0.0082) from the pre- to the peri-COVID-19 pandemic period (Page 4).
-Additionally, the stillbirth rate also increased from 24.4 to 27.1 per 1,000 births during the same period (Page 4). 
-This increase might be due to maternal illness directly linked to COVID-19 infection or indirect consequences of disruptions in health services and other secondary effects induced by the pandemic (Page 5). 
-It's also worth noting that the overwhelming effects of the COVID-19 pandemic could lead to 31% additional maternal and newborn deaths due to reduced access to essential services (Page 2).</t>
+The maternal mortality ratio showed a statistically significant increase from 195 to 230 per 100,000 live births (p = 0.0082) from the pre- to the peri-COVID-19 pandemic period. (Page 4)
+Additionally, it increased from 179.6 to 185.9 per 100,000 live births during the peri-COVID-19 pandemic period (Page 4). 
+This increase may be due to maternal illness directly linked to COVID-19 infection or disruptions in health services (Page 5). 
+The pandemic could lead to 31% additional maternal and newborn deaths due to reduced access to essential services (Page 2).</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -739,13 +744,13 @@
         <v>0.9</v>
       </c>
       <c r="F8" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="G8" t="n">
         <v>0.8</v>
       </c>
       <c r="H8" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="9">
@@ -762,10 +767,9 @@
       <c r="C9" t="inlineStr">
         <is>
           <t>The C-section rate increased during the COVID-19 pandemic.
-According to the text: 
-- "the C-section rate increased from 17.5% to 20.2% (p &lt; 0.001) during the same period" (Page 4).
-- This increase might be attributed to various factors, including alterations in labor and delivery procedures, hospitals adopting new protocols aimed at limiting access to labor-inducing methods, and expectant mothers choosing C-sections out of concern for contracting COVID-19 in hospital environments (Page 6). 
-- Additionally, the use of C-section was mentioned as one of the few RMNCAH indicators that increased during the pandemic (Page 5).</t>
+Specifically, the C-section rate increased from 17.5% to 20.2% (p &lt; 0.001) during the pandemic period (Page 4).
+This trend may be attributed to factors such as alterations in labor and delivery procedures, concerns about contracting COVID-19 in hospital environments, and increased reliance on surgical interventions (Page 6). 
+Additionally, only a small number of indicators, including the rate of C-section, increased during the pandemic (Page 5).</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -778,13 +782,13 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="F9" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
       <c r="G9" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="H9" t="n">
         <v>0.6</v>
@@ -804,10 +808,10 @@
       <c r="C10" t="inlineStr">
         <is>
           <t>The child health indicators that improved despite the pandemic are:
-* Institutional live births beneficiaries of the kangaroo mother care method (increased from 8.6% to 10.4%, p &lt; 0.001)
-* Home visits/postnatal follow-up during days 0–3 (increased from 36.8% to 40.0%, p &lt; 0.001)
-* Pneumococcal conjugate vaccine (increased by over 4 percentage points)
-These indicators showed a statistically significant increase during the peri-COVID-19 pandemic period. (Page 4 and Page 1)</t>
+1. **Institutional live births beneficiaries of the kangaroo mother care method**: increased from 8.6% to 10.4% (p &lt; 0.001) (Page 4)
+2. **Home visits/postnatal follow-up during days 0–3**: increased from 36.8% to 40.0% (p &lt; 0.001) (Page 4)
+3. **Pneumococcal conjugate vaccine uptake**: increased by over 4 percentage points (Pages 1 and 4)
+These indicators showed a statistically significant increase during the pandemic period, indicating an improvement in child health services despite the challenges posed by the pandemic.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -823,7 +827,7 @@
         <v>0.9</v>
       </c>
       <c r="F10" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="G10" t="n">
         <v>0.8</v>
@@ -845,18 +849,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>External factors that may have influenced RMNCAH services in Haiti, besides COVID-19, include:
-* Sociopolitical crisis (Page 1)
-* Control exercised by armed groups over the population (Page 1)
-* Political unrest (Page 6)
-* Violent protests (Page 6)
-* National lockdowns (Page 6)
-* Armed gang activities (Page 6)
-* Frequent kidnappings (Page 6)
-* Economic crisis (Page 6)
-* Corruption (Page 6)
-* Natural events (Page 6)
-These factors may have contributed to the decline observed in RMNCAH services in Haiti, alongside the COVID-19 pandemic. (Page 1 and Page 6)</t>
+          <t>Several external factors, besides COVID-19, may have influenced RMNCAH services in Haiti:
+1. **Sociopolitical crisis**: The country has been experiencing a deep sociopolitical and economic crisis, which may have impacted RMNCAH services (Page 1).
+2. **Armed gang activities and control**: Armed groups have been exerting control over the population, which could have disrupted essential RMNCAH services (Page 1).
+3. **Political unrest and violent protests**: These events have led to national lockdowns, which might have affected the delivery of RMNCAH services (Page 6).
+4. **Frequent kidnappings**: This could have caused disruptions in essential RMNCAH services (Page 6).
+5. **Natural events**: Haiti has been affected by natural events, which may have negatively impacted the SISNU–DHIS2 reporting system and RMNCAH services (Page 6).
+6. **Corruption**: The country's healthcare system has been ravaged by corruption, which could have affected the delivery of RMNCAH services (Page 6).
+These factors may have contributed to the decline observed in RMNCAH services in Haiti, alongside the COVID-19 pandemic.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -894,8 +894,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Heart regeneration is a major focus in medicine because the death of cardiac myocytes leads to diminished heart pump function, causing heart failure, which is a dominant cause of death worldwide. Currently, there are no therapies that directly address the loss of cardiac myocytes, except for transplantation. Therefore, researchers are excited about cardiac regeneration as a potential therapeutic approach to address heart failure. 
-This is supported by the text: "The death of cardiac myocytes diminishes the heart’s pump function and is a major cause of heart failure, one of the dominant causes of death worldwide. Other than transplantation, there are no therapies that directly address the loss of cardiac myocytes, which explains the current excitement in cardiac regeneration." (Page 1)</t>
+          <t>Heart regeneration is a major focus in medicine because:
+1. **Cardiac myocyte death leads to heart failure**: The death of cardiac myocytes diminishes the heart's pump function, causing heart failure, which is a dominant cause of death worldwide (Document: regeneration, Page 1).
+2. **Limited treatment options**: Currently, there are no therapies that directly address the loss of cardiac myocytes, except for transplantation (Document: regeneration, Page 1).
+3. **Potential for improved treatment**: Researchers believe that understanding endogenous cardiac regeneration and developing therapeutic interventions could provide new treatment options for heart failure (Document: regeneration, Page 1).
+Overall, the goal of heart regeneration research is to find alternative treatments for heart failure, which is a significant public health concern.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -933,8 +936,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The traditional belief about the mammalian heart was that it is a terminally differentiated organ, incapable of replenishing any myocyte attrition. 
-This is supported by the text: "Until recently, the prospect of cardiac regeneration was largely a subject of science fiction. The longstanding paradigm held that the mammalian heart is a terminally differentiated organ, incapable of replenishing any myocyte attrition." (Page 1)</t>
+          <t>The traditional belief about the mammalian heart was that it is a **terminally differentiated organ, incapable of replenishing any myocyte attrition** (Document: regeneration, Page 1). This longstanding paradigm held that the mammalian heart lacks the ability to regenerate or replace damaged or lost cardiac myocytes.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -950,7 +952,7 @@
         <v>0.9</v>
       </c>
       <c r="F13" t="n">
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="G13" t="n">
         <v>0.8</v>
@@ -973,11 +975,9 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>Lower organisms that show natural heart regeneration include:
-* Zebraﬁsh 
-* Newts 
-These organisms demonstrate a remarkable survival capacity after removal of up to 20% of the heart by transection of the ventricular apex (Oberpriller &amp; Oberpriller, 1974; Poss et al, 2002). 
-This is supported by the text: 
-"The regenerative deﬁcit of the mammalian heart is obvious when compared with organisms such as zebraﬁsh and newts, which demonstrate a remarkable survival capacity after removal of up to 20% of the heart by transection of the ventricular apex (Oberpriller &amp; Oberpriller, 1974; Poss et al, 2002)." (Page 2)</t>
+1. **Zebrafish**: Studies have demonstrated that zebrafish have a remarkable survival capacity after removal of up to 20% of the heart by transection of the ventricular apex (Poss et al, 2002; Jopling et al, 2010).
+2. **Newts**: Like zebrafish, newts have also been shown to have the ability to regenerate their heart tissue (Oberpriller &amp; Oberpriller, 1974).
+These organisms demonstrate a remarkable capacity for heart regeneration, which is attributed to the ability of pre-existing cardiac myocytes to undergo dedifferentiation, proliferation, and functional integration with the pre-existing myocardium.</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -999,7 +999,7 @@
         <v>0.8</v>
       </c>
       <c r="H14" t="n">
-        <v>0.95</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="15">
@@ -1016,11 +1016,10 @@
       <c r="C15" t="inlineStr">
         <is>
           <t>The mechanisms underlying zebrafish heart regeneration involve:
-1. **Dedifferentiation**: Pre-existing cardiac myocytes adjacent to the injury site undergo dedifferentiation, characterized by the dissolution of sarcomeric structures.
-2. **Proliferation**: These dedifferentiated cardiac myocytes then incorporate DNA synthesis markers, consistent with proliferation.
+1. **Dedifferentiation**: Pre-existing cardiac myocytes adjacent to the injury site undergo dedifferentiation, characterized by dissolution of sarcomeric structures.
+2. **Proliferation**: This is followed by incorporation of DNA synthesis markers, indicating proliferation of cardiac myocytes.
 3. **Functional integration**: Newly generated cardiac myocytes are functionally integrated with the pre-existing myocardium.
-This process is supported by studies, including Jopling et al. (2010), Kikuchi et al. (2010), and Laube et al. (2006). Specifically, Kikuchi et al. (2010) showed that gata4(+) cardiomyocytes make a primary contribution to zebrafish heart regeneration. 
-These findings provide insights into the mechanisms that enable zebrafish to regenerate their hearts, and may have implications for the development of therapeutic approaches to promote heart regeneration in mammals.</t>
+According to studies, gata4(+) cardiomyocytes are primarily responsible for zebrafish heart regeneration (Kikuchi et al, 2010). Additionally, research suggests that zebrafish heart regeneration occurs through cardiomyocyte dedifferentiation and proliferation (Jopling et al, 2010).</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1039,10 +1038,10 @@
         <v>0.95</v>
       </c>
       <c r="G15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H15" t="n">
         <v>0.85</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.8</v>
       </c>
     </row>
     <row r="16">
@@ -1058,20 +1057,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>There is limited evidence suggesting that the mammalian heart has some capacity for cardiac myocyte turnover and regeneration, but the scope of this capacity is still a topic of controversy.
- Studies have reported:
-* The presence of mitotic cardiac myocytes (Kajstura et al, 1998)
-* Immuno-detection of cell cycle markers such as Ki67 (Beltrami et al, 2001)
-* IdU incorporation into newly synthesized DNA (Kajstura et al, 2010b)
-These findings suggest that nearly 30% of the heart can be replaced within 1 year during normal homeostasis, a rate that increases 50-fold after injury (Kajstura et al, 2010b). However, it is unclear whether this regenerative capacity is sufficient for complete heart regeneration.
-Additionally, some studies have shown that neonatal mouse hearts have a transient regenerative potential (Porrello et al, 2011). There is also evidence of chimerism in transplanted hearts, suggesting that some degree of cardiac cell replacement can occur (Quaini et al, 2002).
-However, more research is needed to fully understand the extent of heart regeneration in mammals. 
+          <t>There is some evidence suggesting that the mammalian heart has a limited capacity for regeneration. Studies have shown that:
+* Nearly 30% of the heart can be replaced within 1 year during normal homeostasis, a rate that increases 50-fold after injury (Kajstura et al, 1998; Beltrami et al, 2001; Kajstura et al, 2010b).
+* The neonatal mouse heart has a transient regenerative potential (Porrello et al, 2011).
+* Bone marrow cells have been shown to regenerate infarcted myocardium (Orlic et al, 2001).
+However, there is still controversy about the scope of the mammalian heart's endogenous regenerative capacity. The extent to which the mammalian heart can regenerate is still unclear and requires further research. 
 References:
-* Kajstura et al, 1998
-* Beltrami et al, 2001
-* Kajstura et al, 2010b
-* Porrello et al, 2011
-* Quaini et al, 2002</t>
+- Kajstura et al (1998)
+- Beltrami et al (2001)
+- Kajstura et al (2010b)
+- Porrello et al (2011)
+- Orlic et al (2001)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1109,19 +1105,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The outcome of cell-based therapies with bone marrow progenitors has been modest improvements in ventricular function and subtle improvements in heart failure symptoms.
- Studies have shown:
-* Modest improvements in ventricular function (Martin-Rendon et al, 2008; Schachinger et al, 2006)
-* Significant improvements in cardiac function and a combined clinical endpoint in the REPAIR-AMI study (Schachinger et al, 2006)
-* Some therapeutic effect even in studies with no detectable transdifferentiation (Balsam et al, 2004)
-However, the experience with cell-based therapies in humans does not support widespread adoption at this time due to:
-* Modest benefits
-* Insufficient safety data
-* Anticipated quality control costs (Page 7)
+          <t>The outcome of cell-based therapies with bone marrow progenitors has shown modest improvements in ventricular function and subtle improvements in heart failure symptoms. 
+According to studies:
+* The REPAIR-AMI study (Schachinger et al, 2006) demonstrated significant improvements in cardiac function and a combined clinical endpoint.
+* Randomized clinical trials have shown modest cell therapy-mediated improvements in ventricular function (Martin-Rendon et al, 2008; Schachinger et al, 2006).
+* However, the benefits are limited, and there is insufficient safety data to support widespread adoption (Balsam et al, 2004; Murry et al, 2004).
+Overall, while cell-based therapies with bone marrow progenitors show some therapeutic effect, their modest benefits and safety concerns limit their current adoption. 
 References:
-* Martin-Rendon et al, 2008
-* Schachinger et al, 2006
-* Balsam et al, 2004</t>
+- Schachinger et al (2006)
+- Martin-Rendon et al (2008)
+- Balsam et al (2004)
+- Murry et al (2004)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1134,16 +1128,16 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="F17" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="G17" t="n">
         <v>0.7</v>
       </c>
       <c r="H17" t="n">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="18">
@@ -1160,15 +1154,11 @@
       <c r="C18" t="inlineStr">
         <is>
           <t>Cellular reprogramming plays a significant role in regeneration, particularly in cardiac regeneration. It has been shown that cellular reprogramming can be used to directly convert non-cardiac cells into functional cardiomyocytes.
- Studies have demonstrated:
-* Direct reprogramming of fibroblasts into functional cardiomyocytes by defined factors (Ieda et al, 2010)
-* This approach has the potential to facilitate the development of regenerative therapies for cardiac tissue
-Additionally, cellular reprogramming may also contribute to the activation and recruitment of endogenous cardiac myocyte progenitors through paracrine signalling pathways, which could amplify endogenous regeneration.
-However, further research is needed to fully understand the role of cellular reprogramming in regeneration and to explore its therapeutic potential.
+* A study by Ieda et al (2010) demonstrated that fibroblasts can be directly reprogrammed into functional cardiomyocytes by defined factors.
+* This approach offers a promising strategy for cardiac regeneration, as it bypasses the need for stem cell transplantation and utilizes readily available cell types.
+However, the field is still evolving, and more research is needed to fully understand the potential of cellular reprogramming in regeneration.
 References:
-* Ieda et al, 2010
-* Loffredo et al, 2011 
-* Balsam et al, 2004; Murry et al, 2004</t>
+- Ieda M, Fu JD, Delgado-Olguin P, Vedantham V, Hayashi Y, Bruneau BG, Srivastava D (2010) Direct reprogramming of fibroblasts into functional cardiomyocytes by defined factors. Cell 142: 375-386</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1206,15 +1196,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>The major barriers to successful cardiac regeneration in humans are not explicitly stated in the provided context. However, based on the information given, some challenges can be inferred:
-* Understanding the mechanistic differences between adult mammals with limited regenerative capacity and organisms with robust cardiac regeneration (e.g., neonatal mice, zebrafish, and newts) 
-* Elucidating the scope of endogenous mammalian regeneration and the scale of the regenerative deficit
-* Developing therapeutic interventions that can amplify endogenous heart regeneration
-* Ensuring the safety and efficacy of exogenous regenerative therapies, such as cell-based therapies and pharmacoregenerative strategies.
-Further research is needed to fully understand the barriers to successful cardiac regeneration in humans. 
+          <t>The major barriers to successful cardiac regeneration in humans include:
+1. **Limited understanding of endogenous mammalian regeneration**: The scope of endogenous mammalian cardiac regeneration and the scale of the regenerative deficit are not well understood.
+2. **Mechanistic differences between adult mammals and organisms with high regenerative capacity**: The differences between adult mammals with limited regenerative capacity and organisms like neonatal mice, zebrafish, and newts that demonstrate unambiguous cardiac myocyte regeneration are not well understood.
+3. **Challenges in cell-based therapies**: Cell-based therapies have shown modest improvements in ventricular function and heart failure symptoms, but their benefits are limited, and there are safety concerns.
+4. **Limited efficacy of systemic growth factor therapy**: Systemic growth factor therapy has potential mitogenic effects on other organs, and local delivery of engineered proteins and small molecules is still a developing area.
+Overall, the field of cardiac regeneration faces significant challenges, including understanding the mechanisms of endogenous regeneration, developing effective cell-based therapies, and overcoming the limitations of current approaches.
 References:
-* Page 1, 9 ( multiple documents) 
-Please provide more context or information to provide a more comprehensive answer.</t>
+- Multiple documents in the context, highlighting the complexities and challenges of cardiac regeneration.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1227,16 +1216,16 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="F19" t="n">
-        <v>0.7</v>
+        <v>0.85</v>
       </c>
       <c r="G19" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="H19" t="n">
-        <v>0.9</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="20">
@@ -1253,14 +1242,16 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>Promising directions for regenerative therapy include:
-1. **Exploiting paracrine signalling**: to amplify the existent endogenous regenerative response (Loffredo et al, 2011)
-2. **Pharmacoregenerative strategies**: using small molecules or protein-based therapies to activate repair mechanisms in the heart, which may be a more practical near-term approach (Page 8)
-3. **Local delivery of engineered proteins and small molecules**: targeting specific survival, growth, and differentiation pathways to promote cardiac repair (Page 9)
-4. **Cell-based therapies with improved understanding**: of the mechanistic differences between adult mammals with limited regenerative capacity and organisms with robust cardiac regeneration (Page 9)
-These directions aim to address the challenges in cardiac regeneration, including the limited success of cell-based therapies and the need for more effective and practical therapeutic approaches. 
+1. **Exploiting paracrine signalling**: Amplifying the existent endogenous regenerative response through paracrine signalling, which may be a more practical near-term approach to promote cardiac repair.
+2. **Local delivery of engineered proteins and small molecules**: Targeting specific survival, growth, and differentiation pathways to promote cardiac regeneration, while minimizing potential mitogenic effects on other organs.
+3. **Cellular reprogramming**: Directly converting non-cardiac cells into functional cardiomyocytes, which offers a promising strategy for cardiac regeneration.
+4. **Therapeutic delivery of progenitor cells**: Facilitating the generation of de novo functional myocardium by delivering progenitor cells that can produce new heart cells.
+These approaches aim to overcome the challenges and limitations of current cardiac regeneration therapies, including cell-based therapies, and may lead to more robust and effective regenerative therapies.
 References:
-* Loffredo et al, 2011
-* Page 8, 9</t>
+- Loffredo et al (2011)
+- Balsam et al (2004)
+- Murry et al (2004)
+- Martin-Rendon et al (2008)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1298,10 +1289,10 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>The most pressing issue for advancing cardiac regeneration research is **identifying consistently supported findings across multiple experimental approaches**. This is crucial to ensure that the results are reliable and can be translated into therapeutic interventions that benefit patients. 
-According to the context, "Perhaps the most important issue in this ﬁeld is identifying which ﬁndings are consistently supported by multiple experimental approaches. Ultimately, the ﬁndings that are easily reproduced by most or all laboratories will most likely beneﬁt patients." (Page 9)
-Additionally, understanding the mechanistic differences between adult mammals with limited regenerative capacity and organisms with robust cardiac regeneration is also a significant challenge that needs to be addressed (Page 9). 
-However, based on the provided context, the former is highlighted as a pressing issue.</t>
+          <t>The most pressing issue for advancing cardiac regeneration research is **identifying consistently supported findings across multiple experimental approaches**. This is crucial to ensure that research advances are reliable, reproducible, and ultimately beneficial to patients.
+According to the context, "Perhaps the most important issue in this field is identifying which findings are consistently supported by multiple experimental approaches. Ultimately, the findings that are easily reproduced by most or all laboratories will most likely benefit patients." (Score: 0.8298471570014954)
+Additionally, understanding the **mechanistic differences between adult mammals and organisms with high regenerative capacity** is also a significant issue, as it may reveal new pathways for therapeutic targeting (Score: 0.8267030715942383). 
+However, the top priority is to identify reliable and reproducible findings to advance the field.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1314,16 +1305,16 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="F21" t="n">
         <v>0.95</v>
       </c>
       <c r="G21" t="n">
-        <v>0.8</v>
+        <v>0.88</v>
       </c>
       <c r="H21" t="n">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>